<commit_message>
docs(sheet-template): add purge URL placeholder to Panduan tab
Add a "Link penting" section at the top of the Panduan guide tab in the
sheet template. Shows the purge URL in the format:
  https://namawebsite.netlify.app/purge?secret=GANTI_INI
with a note to replace the domain and secret with the real values
provided by the developer, and explains the 1–2 min cache window.

Regenerated docs/kozy-sheet-template.xlsx from the updated script.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ENxJBzSCVwTaatiy7EeHne
</commit_message>
<xml_diff>
--- a/docs/kozy-sheet-template.xlsx
+++ b/docs/kozy-sheet-template.xlsx
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C48"/>
+  <dimension ref="B2:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -728,7 +728,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tab yang dibaca website</t>
+          <t>Link penting</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -736,402 +736,423 @@
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>config</t>
+          <t>Perbarui website</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Nama properti, kalimat perkenalan, nomor WhatsApp utama, dan alamat kantor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>lokasi</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Satu baris untuk satu bangunan kos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>kamar</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Satu baris untuk satu kamar fisik. Baris inilah yang jadi kotak di denah kamar.</t>
-        </is>
-      </c>
+          <t>https://namawebsite.netlify.app/purge?secret=GANTI_INI
+Ganti namawebsite dan GANTI_INI dengan URL dan rahasia yang diberikan developer. Simpan sebagai bookmark. Buka link ini setiap kali mengubah data di Sheet supaya perubahan langsung muncul. Tanpa dibuka pun perubahan muncul sendiri dalam 1–2 menit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tab yang dibaca website</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>denah</t>
+          <t>config</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Opsional. Menggambar tata letak tiap lantai. Kalau dikosongkan, denah kamar tetap tampil sebagai daftar kotak per lantai.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Menggambar denah lantai (opsional)</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr"/>
+          <t>Nama properti, kalimat perkenalan, nomor WhatsApp utama, dan alamat kantor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>lokasi</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Satu baris untuk satu bangunan kos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>kamar</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Satu baris untuk satu kamar fisik. Baris inilah yang jadi kotak di denah kamar.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Satu baris = satu baris denah</t>
+          <t>denah</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Di tab denah, isi lokasi_slug, lantai, dan baris (1, 2, 3 dari depan ke belakang).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Kolom sel</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Tulis isi kotak dari kiri ke kanan, dipisah koma. Contoh: A1, A2, lorong, A3, tangga.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Kata kunci</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>pintu, tangga, lift, lorong tampil dengan ikon. Titik (.) berarti kotak kosong.</t>
-        </is>
-      </c>
+          <t>Opsional. Menggambar tata letak tiap lantai. Kalau dikosongkan, denah kamar tetap tampil sebagai daftar kotak per lantai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Menggambar denah lantai (opsional)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Tulisan bebas</t>
+          <t>Satu baris = satu baris denah</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Kata lain seperti WC atau Dapur tampil apa adanya sebagai penanda.</t>
+          <t>Di tab denah, isi lokasi_slug, lantai, dan baris (1, 2, 3 dari depan ke belakang).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>arah</t>
+          <t>Kolom sel</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Boleh dikosongkan. Isi utara / selatan / timur / barat di salah satu baris lantai untuk menampilkan kompas.</t>
+          <t>Tulis isi kotak dari kiri ke kanan, dipisah koma. Contoh: A1, A2, lorong, A3, tangga.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Salah ketik aman</t>
+          <t>Kata kunci</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Kode kamar yang tidak dikenali tidak hilang, kamarnya muncul di bagian Belum dipetakan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Mengubah status kamar</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr"/>
+          <t>pintu, tangga, lift, lorong tampil dengan ikon. Titik (.) berarti kotak kosong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Tulisan bebas</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Kata lain seperti WC atau Dapur tampil apa adanya sebagai penanda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>arah</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Boleh dikosongkan. Isi utara / selatan / timur / barat di salah satu baris lantai untuk menampilkan kompas.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>Salah ketik aman</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Kode kamar yang tidak dikenali tidak hilang, kamarnya muncul di bagian Belum dipetakan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Mengubah status kamar</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Buka tab kamar, cari baris kamarnya lewat kolom kode.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Ketuk kolom status, pilih kosong, dibooking, atau terisi dari dropdown.</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Buka bookmark Perbarui website. Tanpa langkah ini pun perubahan muncul sendiri dalam 5 menit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Menambah tipe kamar</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Tidak ada tab tipe</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Tipe kamar terbentuk sendiri dari kolom tipe di tab kamar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Tulis sama persis</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Deluxe AC dan Deluxe A/C dianggap dua tipe berbeda. Pakai dropdown supaya seragam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Samakan isinya</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Harga, luas, dan fasilitas semua kamar bertipe sama sebaiknya diisi sama.</t>
-        </is>
-      </c>
+          <t>Buka bookmark Perbarui website. Tanpa langkah ini pun perubahan muncul sendiri dalam 5 menit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Menambah tipe kamar</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Fasilitas dipotong</t>
+          <t>Tidak ada tab tipe</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Kartu tipe hanya menampilkan fasilitas yang dimiliki SEMUA kamar bertipe itu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Menambah lokasi</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr"/>
+          <t>Tipe kamar terbentuk sendiri dari kolom tipe di tab kamar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Tulis sama persis</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Deluxe AC dan Deluxe A/C dianggap dua tipe berbeda. Pakai dropdown supaya seragam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Samakan isinya</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Harga, luas, dan fasilitas semua kamar bertipe sama sebaiknya diisi sama.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Fasilitas dipotong</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Tab lokasi, tambah baris. Isi minimal slug, nama, alamat, dan aktif = TRUE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Kolom nomor_wa boleh dikosongkan kalau lokasi ini memakai nomor utama di tab config.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Tab kamar, tambah baris kamarnya. Kolom lokasi_slug pilih dari dropdown.</t>
-        </is>
-      </c>
+          <t>Kartu tipe hanya menampilkan fasilitas yang dimiliki SEMUA kamar bertipe itu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Menambah lokasi</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Buka bookmark Perbarui website. Halaman /locations/{slug} langsung ada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Yang tidak boleh dilakukan</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr"/>
+          <t>Tab lokasi, tambah baris. Isi minimal slug, nama, alamat, dan aktif = TRUE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Kolom nomor_wa boleh dikosongkan kalau lokasi ini memakai nomor utama di tab config.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Tab kamar, tambah baris kamarnya. Kolom lokasi_slug pilih dari dropdown.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Jangan hapus baris</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Untuk menyembunyikan lokasi atau kamar, ubah kolom aktif menjadi FALSE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Jangan ubah baris 1</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Nama kolom di baris pertama dipakai website untuk mengenali datanya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Jangan ubah nama tab</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>config, lokasi, dan kamar harus tetap bernama persis itu, huruf kecil. Tab denah opsional, tetapi kalau dipakai namanya juga harus denah.</t>
-        </is>
-      </c>
+          <t>Buka bookmark Perbarui website. Halaman /locations/{slug} langsung ada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Yang tidak boleh dilakukan</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Jangan cabut sharing</t>
+          <t>Jangan hapus baris</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>File harus tetap Anyone with the link, Viewer. Kalau dicabut, website memakai data cadangan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Melihat angka terbaru</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr"/>
+          <t>Untuk menyembunyikan lokasi atau kamar, ubah kolom aktif menjadi FALSE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Jangan ubah baris 1</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Nama kolom di baris pertama dipakai website untuk mengenali datanya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Jangan ubah nama tab</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>config, lokasi, dan kamar harus tetap bernama persis itu, huruf kecil. Tab denah opsional, tetapi kalau dipakai namanya juga harus denah.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="B43" s="4" t="inlineStr">
         <is>
+          <t>Jangan cabut sharing</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>File harus tetap Anyone with the link, Viewer. Kalau dicabut, website memakai data cadangan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Melihat angka terbaru</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>Halaman depan menampilkan jumlah lokasi, total kamar kosong, dan harga terendah.</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Halaman lokasi</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Denah kamar menampilkan status tiap kamar, dikelompokkan per lantai.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>Kalau ada yang aneh</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="B47" s="4" t="inlineStr">
         <is>
+          <t>Halaman lokasi</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Denah kamar menampilkan status tiap kamar, dikelompokkan per lantai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Kalau ada yang aneh</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
           <t>Buka /purge</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>Halaman itu menyebut sumber data yang sedang dipakai, jumlah baris terbaca, dan baris mana yang dilewati karena datanya belum lengkap.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="B48" s="4" t="inlineStr">
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Website tidak pernah kosong</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Kalau Sheet bermasalah, yang tampil adalah data terakhir yang tersimpan di kode.</t>
         </is>

</xml_diff>

<commit_message>
feat(deploy): migrate hosting from Netlify to Vercel (#3)
Replaces the Netlify adapter with a Node-to-Web handler in api/index.mjs,
since TanStack Start ships no Vercel target. Netlify Blobs has no Vercel
equivalent, so the build now bakes a Sheet snapshot into the server bundle
as the last-resort fallback, emitted only when the build genuinely read the
Sheet. Purge clears the server cache and lets the 60s edge TTL expire rather
than invalidating by CDN tag.

Also rewrites the README as a concise setup guide and regenerates the lock
file to fix npm ci.
</commit_message>
<xml_diff>
--- a/docs/kozy-sheet-template.xlsx
+++ b/docs/kozy-sheet-template.xlsx
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C48"/>
+  <dimension ref="B2:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -728,7 +728,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tab yang dibaca website</t>
+          <t>Link penting</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -736,402 +736,423 @@
     <row r="6" ht="30" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>config</t>
+          <t>Perbarui website</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Nama properti, kalimat perkenalan, nomor WhatsApp utama, dan alamat kantor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>lokasi</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Satu baris untuk satu bangunan kos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>kamar</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Satu baris untuk satu kamar fisik. Baris inilah yang jadi kotak di denah kamar.</t>
-        </is>
-      </c>
+          <t>https://namawebsite.vercel.app/purge?secret=GANTI_INI
+Ganti namawebsite dan GANTI_INI dengan URL dan rahasia yang diberikan developer. Simpan sebagai bookmark. Buka link ini setiap kali mengubah data di Sheet supaya perubahan langsung muncul. Tanpa dibuka pun perubahan muncul sendiri dalam 1–2 menit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tab yang dibaca website</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>denah</t>
+          <t>config</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Opsional. Menggambar tata letak tiap lantai. Kalau dikosongkan, denah kamar tetap tampil sebagai daftar kotak per lantai.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Menggambar denah lantai (opsional)</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr"/>
+          <t>Nama properti, kalimat perkenalan, nomor WhatsApp utama, dan alamat kantor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>lokasi</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Satu baris untuk satu bangunan kos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>kamar</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Satu baris untuk satu kamar fisik. Baris inilah yang jadi kotak di denah kamar.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Satu baris = satu baris denah</t>
+          <t>denah</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Di tab denah, isi lokasi_slug, lantai, dan baris (1, 2, 3 dari depan ke belakang).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Kolom sel</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Tulis isi kotak dari kiri ke kanan, dipisah koma. Contoh: A1, A2, lorong, A3, tangga.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Kata kunci</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>pintu, tangga, lift, lorong tampil dengan ikon. Titik (.) berarti kotak kosong.</t>
-        </is>
-      </c>
+          <t>Opsional. Menggambar tata letak tiap lantai. Kalau dikosongkan, denah kamar tetap tampil sebagai daftar kotak per lantai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Menggambar denah lantai (opsional)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Tulisan bebas</t>
+          <t>Satu baris = satu baris denah</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Kata lain seperti WC atau Dapur tampil apa adanya sebagai penanda.</t>
+          <t>Di tab denah, isi lokasi_slug, lantai, dan baris (1, 2, 3 dari depan ke belakang).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>arah</t>
+          <t>Kolom sel</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Boleh dikosongkan. Isi utara / selatan / timur / barat di salah satu baris lantai untuk menampilkan kompas.</t>
+          <t>Tulis isi kotak dari kiri ke kanan, dipisah koma. Contoh: A1, A2, lorong, A3, tangga.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Salah ketik aman</t>
+          <t>Kata kunci</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Kode kamar yang tidak dikenali tidak hilang, kamarnya muncul di bagian Belum dipetakan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Mengubah status kamar</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr"/>
+          <t>pintu, tangga, lift, lorong tampil dengan ikon. Titik (.) berarti kotak kosong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Tulisan bebas</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Kata lain seperti WC atau Dapur tampil apa adanya sebagai penanda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>arah</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Boleh dikosongkan. Isi utara / selatan / timur / barat di salah satu baris lantai untuk menampilkan kompas.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>Salah ketik aman</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Kode kamar yang tidak dikenali tidak hilang, kamarnya muncul di bagian Belum dipetakan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Mengubah status kamar</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Buka tab kamar, cari baris kamarnya lewat kolom kode.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="4" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Ketuk kolom status, pilih kosong, dibooking, atau terisi dari dropdown.</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Buka bookmark Perbarui website. Tanpa langkah ini pun perubahan muncul sendiri dalam 5 menit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Menambah tipe kamar</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Tidak ada tab tipe</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Tipe kamar terbentuk sendiri dari kolom tipe di tab kamar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Tulis sama persis</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Deluxe AC dan Deluxe A/C dianggap dua tipe berbeda. Pakai dropdown supaya seragam.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Samakan isinya</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Harga, luas, dan fasilitas semua kamar bertipe sama sebaiknya diisi sama.</t>
-        </is>
-      </c>
+          <t>Buka bookmark Perbarui website. Tanpa langkah ini pun perubahan muncul sendiri dalam 5 menit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Menambah tipe kamar</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Fasilitas dipotong</t>
+          <t>Tidak ada tab tipe</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Kartu tipe hanya menampilkan fasilitas yang dimiliki SEMUA kamar bertipe itu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Menambah lokasi</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr"/>
+          <t>Tipe kamar terbentuk sendiri dari kolom tipe di tab kamar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Tulis sama persis</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Deluxe AC dan Deluxe A/C dianggap dua tipe berbeda. Pakai dropdown supaya seragam.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Samakan isinya</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Harga, luas, dan fasilitas semua kamar bertipe sama sebaiknya diisi sama.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Fasilitas dipotong</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Tab lokasi, tambah baris. Isi minimal slug, nama, alamat, dan aktif = TRUE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Kolom nomor_wa boleh dikosongkan kalau lokasi ini memakai nomor utama di tab config.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Tab kamar, tambah baris kamarnya. Kolom lokasi_slug pilih dari dropdown.</t>
-        </is>
-      </c>
+          <t>Kartu tipe hanya menampilkan fasilitas yang dimiliki SEMUA kamar bertipe itu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Menambah lokasi</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Buka bookmark Perbarui website. Halaman /locations/{slug} langsung ada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Yang tidak boleh dilakukan</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr"/>
+          <t>Tab lokasi, tambah baris. Isi minimal slug, nama, alamat, dan aktif = TRUE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Kolom nomor_wa boleh dikosongkan kalau lokasi ini memakai nomor utama di tab config.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Tab kamar, tambah baris kamarnya. Kolom lokasi_slug pilih dari dropdown.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Jangan hapus baris</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Untuk menyembunyikan lokasi atau kamar, ubah kolom aktif menjadi FALSE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Jangan ubah baris 1</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>Nama kolom di baris pertama dipakai website untuk mengenali datanya.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Jangan ubah nama tab</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>config, lokasi, dan kamar harus tetap bernama persis itu, huruf kecil. Tab denah opsional, tetapi kalau dipakai namanya juga harus denah.</t>
-        </is>
-      </c>
+          <t>Buka bookmark Perbarui website. Halaman /locations/{slug} langsung ada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Yang tidak boleh dilakukan</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Jangan cabut sharing</t>
+          <t>Jangan hapus baris</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>File harus tetap Anyone with the link, Viewer. Kalau dicabut, website memakai data cadangan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Melihat angka terbaru</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr"/>
+          <t>Untuk menyembunyikan lokasi atau kamar, ubah kolom aktif menjadi FALSE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Jangan ubah baris 1</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Nama kolom di baris pertama dipakai website untuk mengenali datanya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Jangan ubah nama tab</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>config, lokasi, dan kamar harus tetap bernama persis itu, huruf kecil. Tab denah opsional, tetapi kalau dipakai namanya juga harus denah.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="B43" s="4" t="inlineStr">
         <is>
+          <t>Jangan cabut sharing</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>File harus tetap Anyone with the link, Viewer. Kalau dicabut, website memakai data cadangan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Melihat angka terbaru</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>Halaman depan menampilkan jumlah lokasi, total kamar kosong, dan harga terendah.</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Halaman lokasi</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Denah kamar menampilkan status tiap kamar, dikelompokkan per lantai.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>Kalau ada yang aneh</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="B47" s="4" t="inlineStr">
         <is>
+          <t>Halaman lokasi</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Denah kamar menampilkan status tiap kamar, dikelompokkan per lantai.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Kalau ada yang aneh</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
           <t>Buka /purge</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>Halaman itu menyebut sumber data yang sedang dipakai, jumlah baris terbaca, dan baris mana yang dilewati karena datanya belum lengkap.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="B48" s="4" t="inlineStr">
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Website tidak pernah kosong</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Kalau Sheet bermasalah, yang tampil adalah data terakhir yang tersimpan di kode.</t>
         </is>

</xml_diff>